<commit_message>
fix: correct battery specifications
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -1,148 +1,463 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\LuwuDynamics\product\XGO_Duck\arduino\xgoduck_hardware\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B66A4D-93C4-497A-9C0A-E179BCE220B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowHeight="16660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>Part Name</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Purchase Link</t>
+  </si>
   <si>
     <t>Arduino Uno q</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://store.arduino.cc/</t>
+  </si>
+  <si>
+    <t>Robot Expansion Board</t>
   </si>
   <si>
     <t>AMP 3Pin Cable</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Robot Expansion Board</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.alibaba.com/product-detail/Microduck-Servo-Kit-Feetech-Low-Cost_1601942207064.html?spm=a2756.order-detail-bn.0.0.6b072fc22OPijK</t>
   </si>
   <si>
     <t>Feetech 1910</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>18650 battery 8.4V</t>
+  </si>
+  <si>
+    <t>XH2.54 Battery capacity &gt; 2,500 mAh; discharge rating &gt; 3C.</t>
   </si>
   <si>
     <t>Countersunk screw  M2*6</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>screw  M2.5*6</t>
   </si>
   <si>
     <t>screw  M3*16</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>screw  M2.5*6</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bearing  10*15*3</t>
   </si>
   <si>
     <t>Bearing  16*22*4</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Bearing  10*15*3</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Index</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Part Name</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Quantity</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Purchase Link</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.alibaba.com/product-detail/Microduck-Servo-Kit-Feetech-Low-Cost_1601942207064.html?spm=a2756.order-detail-bn.0.0.6b072fc22OPijK</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">18650 battery 8.4V </t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://store.arduino.cc/</t>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Microsoft YaHei"/>
-      <family val="2"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="等线"/>
-      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="等线"/>
-      <family val="3"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
-      <color theme="10"/>
-      <name val="等线"/>
-      <family val="2"/>
+      <color rgb="FF800080"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -191,10 +506,249 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -207,35 +761,78 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="超链接" xfId="1" builtinId="8"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
@@ -251,27 +848,21 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="图片 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17FDF93E-31A1-244B-C934-AE97FE7B8B98}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
+        <xdr:cNvPr id="3" name="图片 2"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="7741919" y="906780"/>
-          <a:ext cx="1234441" cy="1279766"/>
+          <a:off x="7214870" y="1082040"/>
+          <a:ext cx="1235075" cy="1279525"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -326,7 +917,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="Yu Gothic Light"/>
@@ -361,7 +952,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="Yu Gothic"/>
@@ -535,37 +1126,32 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
-    <col min="2" max="2" width="57.88671875" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" customWidth="1"/>
-    <col min="4" max="4" width="70.77734375" customWidth="1"/>
+    <col min="2" max="2" width="57.8839285714286" customWidth="1"/>
+    <col min="3" max="3" width="8.85714285714286" customWidth="1"/>
+    <col min="4" max="4" width="148.428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -573,13 +1159,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C2" s="3">
         <v>1</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>15</v>
+      <c r="D2" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -587,7 +1173,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3">
         <v>1</v>
@@ -599,13 +1185,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C4" s="3">
         <v>15</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>13</v>
+      <c r="D4" s="5" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -613,31 +1199,33 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C5" s="3">
         <v>15</v>
       </c>
-      <c r="D5" s="5"/>
+      <c r="D5" s="6"/>
     </row>
-    <row r="6" spans="1:4" ht="105.6" customHeight="1">
+    <row r="6" ht="105.6" customHeight="1" spans="1:4">
       <c r="A6" s="3">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C6" s="3">
         <v>1</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="3">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C7" s="3">
         <v>200</v>
@@ -649,7 +1237,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C8" s="3">
         <v>6</v>
@@ -661,7 +1249,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C9" s="3">
         <v>4</v>
@@ -673,7 +1261,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C10" s="3">
         <v>2</v>
@@ -685,7 +1273,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C11" s="3">
         <v>11</v>
@@ -696,13 +1284,13 @@
   <mergeCells count="1">
     <mergeCell ref="D4:D5"/>
   </mergeCells>
-  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="D4" r:id="rId1" xr:uid="{8580AEAE-815D-4B3D-A9CA-89BAA2EBD32F}"/>
-    <hyperlink ref="D2" r:id="rId2" xr:uid="{2746B9A3-01D9-4743-83ED-10528885E10E}"/>
+    <hyperlink ref="D4" r:id="rId2" display="https://www.alibaba.com/product-detail/Microduck-Servo-Kit-Feetech-Low-Cost_1601942207064.html?spm=a2756.order-detail-bn.0.0.6b072fc22OPijK"/>
+    <hyperlink ref="D2" r:id="rId3" display="https://store.arduino.cc/"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
-  <drawing r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add 8.4 V Li-ion charger with DC5521 plug to BOM
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Index</t>
   </si>
@@ -41,7 +41,7 @@
     <t>Purchase Link</t>
   </si>
   <si>
-    <t>Arduino Uno q</t>
+    <t>Arduino UnoQ</t>
   </si>
   <si>
     <t>https://store.arduino.cc/</t>
@@ -65,19 +65,22 @@
     <t>XH2.54 Battery capacity &gt; 2,500 mAh; discharge rating &gt; 3C.</t>
   </si>
   <si>
-    <t>Countersunk screw  M2*6</t>
-  </si>
-  <si>
-    <t>screw  M2.5*6</t>
-  </si>
-  <si>
-    <t>screw  M3*16</t>
-  </si>
-  <si>
-    <t>Bearing  10*15*3</t>
-  </si>
-  <si>
-    <t>Bearing  16*22*4</t>
+    <t>8.4 V Li-ion Battery Charger with 5.5 × 2.1 mm DC Barrel Plug (DC5521)</t>
+  </si>
+  <si>
+    <t>Countersunk screw M2*6</t>
+  </si>
+  <si>
+    <t>screw M2.5*6</t>
+  </si>
+  <si>
+    <t>screw M3*16</t>
+  </si>
+  <si>
+    <t>Bearing 10*15*3</t>
+  </si>
+  <si>
+    <t>Bearing 16*22*4</t>
   </si>
 </sst>
 </file>
@@ -90,7 +93,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,13 +118,6 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -607,146 +603,146 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -861,7 +857,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="10800000">
-          <a:off x="7214870" y="1082040"/>
+          <a:off x="7919085" y="1082040"/>
           <a:ext cx="1235075" cy="1279525"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1132,10 +1128,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
-    <col min="2" max="2" width="57.8839285714286" customWidth="1"/>
+    <col min="2" max="2" width="67.7857142857143" customWidth="1"/>
     <col min="3" max="3" width="8.85714285714286" customWidth="1"/>
     <col min="4" max="4" width="148.428571428571" customWidth="1"/>
   </cols>
@@ -1228,7 +1224,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="3">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="D7" s="3"/>
     </row>
@@ -1240,7 +1236,7 @@
         <v>13</v>
       </c>
       <c r="C8" s="3">
-        <v>6</v>
+        <v>200</v>
       </c>
       <c r="D8" s="3"/>
     </row>
@@ -1252,7 +1248,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D9" s="3"/>
     </row>
@@ -1264,7 +1260,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D10" s="3"/>
     </row>
@@ -1276,9 +1272,21 @@
         <v>16</v>
       </c>
       <c r="C11" s="3">
+        <v>2</v>
+      </c>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="B12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="3">
+        <v>11</v>
+      </c>
+      <c r="D12" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(bom): Add driver board purchase link
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Index</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>Robot Expansion Board</t>
+  </si>
+  <si>
+    <t>https://shop.xgorobot.com/products/robot-driver-board?variant=67594424713467</t>
   </si>
   <si>
     <t>AMP 3Pin Cable</t>
@@ -1174,20 +1177,22 @@
       <c r="C3" s="3">
         <v>1</v>
       </c>
-      <c r="D3" s="3"/>
+      <c r="D3" s="4" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="3">
         <v>15</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1195,7 +1200,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" s="3">
         <v>15</v>
@@ -1207,13 +1212,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3">
         <v>1</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1221,7 +1226,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
@@ -1233,7 +1238,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="3">
         <v>200</v>
@@ -1245,7 +1250,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" s="3">
         <v>6</v>
@@ -1257,7 +1262,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" s="3">
         <v>4</v>
@@ -1269,7 +1274,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11" s="3">
         <v>2</v>
@@ -1281,7 +1286,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C12" s="3">
         <v>11</v>
@@ -1295,6 +1300,7 @@
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId2" display="https://www.alibaba.com/product-detail/Microduck-Servo-Kit-Feetech-Low-Cost_1601942207064.html?spm=a2756.order-detail-bn.0.0.6b072fc22OPijK"/>
     <hyperlink ref="D2" r:id="rId3" display="https://store.arduino.cc/"/>
+    <hyperlink ref="D3" r:id="rId4" display="https://shop.xgorobot.com/products/robot-driver-board?variant=67594424713467"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>